<commit_message>
Update CSV, XLSX, and Google Sheet reports
</commit_message>
<xml_diff>
--- a/minio-report-tracker/xlxs/cellbox21.xlsx
+++ b/minio-report-tracker/xlxs/cellbox21.xlsx
@@ -356,81 +356,6 @@
     </pic>
     <clientData/>
   </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>198</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="7620000" cy="3810000"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="10" name="Image 10" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId10"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>220</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="7620000" cy="3810000"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="11" name="Image 11" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId11"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>242</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="7620000" cy="3810000"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="12" name="Image 12" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId12"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
 </wsDr>
 </file>
 
@@ -723,51 +648,51 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR13"/>
+  <dimension ref="A1:AR10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="5" customWidth="1" min="3" max="3"/>
+    <col width="6" customWidth="1" min="3" max="3"/>
     <col width="5" customWidth="1" min="4" max="4"/>
-    <col width="5" customWidth="1" min="5" max="5"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
     <col width="5" customWidth="1" min="6" max="6"/>
-    <col width="5" customWidth="1" min="7" max="7"/>
-    <col width="5" customWidth="1" min="8" max="8"/>
+    <col width="4" customWidth="1" min="7" max="7"/>
+    <col width="4" customWidth="1" min="8" max="8"/>
     <col width="2" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="5" customWidth="1" min="12" max="12"/>
+    <col width="6" customWidth="1" min="12" max="12"/>
     <col width="5" customWidth="1" min="13" max="13"/>
-    <col width="5" customWidth="1" min="14" max="14"/>
+    <col width="6" customWidth="1" min="14" max="14"/>
     <col width="5" customWidth="1" min="15" max="15"/>
-    <col width="5" customWidth="1" min="16" max="16"/>
-    <col width="5" customWidth="1" min="17" max="17"/>
+    <col width="4" customWidth="1" min="16" max="16"/>
+    <col width="4" customWidth="1" min="17" max="17"/>
     <col width="2" customWidth="1" min="18" max="18"/>
-    <col width="18" customWidth="1" min="19" max="19"/>
+    <col width="15" customWidth="1" min="19" max="19"/>
     <col width="16" customWidth="1" min="20" max="20"/>
     <col width="6" customWidth="1" min="21" max="21"/>
-    <col width="6" customWidth="1" min="22" max="22"/>
-    <col width="5" customWidth="1" min="23" max="23"/>
+    <col width="5" customWidth="1" min="22" max="22"/>
+    <col width="6" customWidth="1" min="23" max="23"/>
     <col width="5" customWidth="1" min="24" max="24"/>
     <col width="4" customWidth="1" min="25" max="25"/>
     <col width="4" customWidth="1" min="26" max="26"/>
     <col width="2" customWidth="1" min="27" max="27"/>
-    <col width="18" customWidth="1" min="28" max="28"/>
+    <col width="15" customWidth="1" min="28" max="28"/>
     <col width="16" customWidth="1" min="29" max="29"/>
     <col width="6" customWidth="1" min="30" max="30"/>
-    <col width="6" customWidth="1" min="31" max="31"/>
-    <col width="5" customWidth="1" min="32" max="32"/>
+    <col width="5" customWidth="1" min="31" max="31"/>
+    <col width="6" customWidth="1" min="32" max="32"/>
     <col width="5" customWidth="1" min="33" max="33"/>
     <col width="4" customWidth="1" min="34" max="34"/>
     <col width="4" customWidth="1" min="35" max="35"/>
     <col width="2" customWidth="1" min="36" max="36"/>
-    <col width="18" customWidth="1" min="37" max="37"/>
+    <col width="15" customWidth="1" min="37" max="37"/>
     <col width="16" customWidth="1" min="38" max="38"/>
     <col width="6" customWidth="1" min="39" max="39"/>
     <col width="6" customWidth="1" min="40" max="40"/>
-    <col width="5" customWidth="1" min="41" max="41"/>
-    <col width="5" customWidth="1" min="42" max="42"/>
+    <col width="4" customWidth="1" min="41" max="41"/>
+    <col width="4" customWidth="1" min="42" max="42"/>
     <col width="4" customWidth="1" min="43" max="43"/>
     <col width="4" customWidth="1" min="44" max="44"/>
   </cols>
@@ -977,22 +902,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>08-December-2025</t>
+          <t>06-March-2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>masterdata-ara</t>
+          <t>auth</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>945</t>
+          <t>612</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>895</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -1002,32 +927,32 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>603</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>05-December-2025</t>
+          <t>05-March-2026</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>masterdata-ara</t>
+          <t>auth</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>945</t>
+          <t>612</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -1037,27 +962,27 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>930</t>
+          <t>0</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>603</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>0</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>9</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>04-December-2025</t>
+          <t>04-March-2026</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -1072,7 +997,7 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>583</t>
+          <t>0</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
@@ -1082,119 +1007,119 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>603</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>03-March-2026</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>auth</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>612</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>603</t>
+        </is>
+      </c>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="AK2" t="inlineStr">
+        <is>
+          <t>02-March-2026</t>
+        </is>
+      </c>
+      <c r="AL2" t="inlineStr">
+        <is>
+          <t>auth</t>
+        </is>
+      </c>
+      <c r="AM2" t="inlineStr">
+        <is>
+          <t>612</t>
+        </is>
+      </c>
+      <c r="AN2" t="inlineStr">
+        <is>
+          <t>598</t>
+        </is>
+      </c>
+      <c r="AO2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AP2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AQ2" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="AB2" t="inlineStr">
-        <is>
-          <t>03-December-2025</t>
-        </is>
-      </c>
-      <c r="AC2" t="inlineStr">
-        <is>
-          <t>auth</t>
-        </is>
-      </c>
-      <c r="AD2" t="inlineStr">
-        <is>
-          <t>612</t>
-        </is>
-      </c>
-      <c r="AE2" t="inlineStr">
-        <is>
-          <t>583</t>
-        </is>
-      </c>
-      <c r="AF2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AG2" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="AH2" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="AI2" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="AK2" t="inlineStr">
-        <is>
-          <t>02-December-2025</t>
-        </is>
-      </c>
-      <c r="AL2" t="inlineStr">
-        <is>
-          <t>auth</t>
-        </is>
-      </c>
-      <c r="AM2" t="inlineStr">
-        <is>
-          <t>612</t>
-        </is>
-      </c>
-      <c r="AN2" t="inlineStr">
-        <is>
-          <t>583</t>
-        </is>
-      </c>
-      <c r="AO2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AP2" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="AQ2" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
       <c r="AR2" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>9</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>08-December-2025</t>
+          <t>06-March-2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>masterdata-eng</t>
+          <t>idrepo</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>945</t>
+          <t>414</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>923</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -1204,7 +1129,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>414</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -1214,22 +1139,22 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>05-December-2025</t>
+          <t>05-March-2026</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>masterdata-eng</t>
+          <t>idrepo</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>945</t>
+          <t>414</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -1239,12 +1164,12 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>945</t>
+          <t>0</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>414</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -1259,7 +1184,7 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>04-December-2025</t>
+          <t>04-March-2026</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -1274,7 +1199,7 @@
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>316</t>
+          <t>0</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
@@ -1284,109 +1209,109 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>414</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>03-March-2026</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>idrepo</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>414</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AF3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AG3" t="inlineStr">
+        <is>
+          <t>414</t>
+        </is>
+      </c>
+      <c r="AH3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AI3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AK3" t="inlineStr">
+        <is>
+          <t>02-March-2026</t>
+        </is>
+      </c>
+      <c r="AL3" t="inlineStr">
+        <is>
+          <t>idrepo</t>
+        </is>
+      </c>
+      <c r="AM3" t="inlineStr">
+        <is>
+          <t>414</t>
+        </is>
+      </c>
+      <c r="AN3" t="inlineStr">
+        <is>
+          <t>336</t>
+        </is>
+      </c>
+      <c r="AO3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AP3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AQ3" t="inlineStr">
+        <is>
           <t>78</t>
         </is>
       </c>
-      <c r="Z3" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="AB3" t="inlineStr">
-        <is>
-          <t>03-December-2025</t>
-        </is>
-      </c>
-      <c r="AC3" t="inlineStr">
-        <is>
-          <t>idrepo</t>
-        </is>
-      </c>
-      <c r="AD3" t="inlineStr">
-        <is>
-          <t>414</t>
-        </is>
-      </c>
-      <c r="AE3" t="inlineStr">
-        <is>
-          <t>315</t>
-        </is>
-      </c>
-      <c r="AF3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AG3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AH3" t="inlineStr">
-        <is>
-          <t>78</t>
-        </is>
-      </c>
-      <c r="AI3" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="AK3" t="inlineStr">
-        <is>
-          <t>02-December-2025</t>
-        </is>
-      </c>
-      <c r="AL3" t="inlineStr">
-        <is>
-          <t>idrepo</t>
-        </is>
-      </c>
-      <c r="AM3" t="inlineStr">
-        <is>
-          <t>414</t>
-        </is>
-      </c>
-      <c r="AN3" t="inlineStr">
-        <is>
-          <t>316</t>
-        </is>
-      </c>
-      <c r="AO3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AP3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AQ3" t="inlineStr">
-        <is>
-          <t>78</t>
-        </is>
-      </c>
       <c r="AR3" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>08-December-2025</t>
+          <t>06-March-2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>masterdata-fra</t>
+          <t>masterdata-ara</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1396,12 +1321,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>907</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>930</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1416,17 +1341,17 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>05-December-2025</t>
+          <t>05-March-2026</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>masterdata-fra</t>
+          <t>masterdata-ara</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -1461,7 +1386,7 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>04-December-2025</t>
+          <t>04-March-2026</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -1476,14 +1401,14 @@
       </c>
       <c r="V4" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
           <t>930</t>
         </is>
       </c>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="X4" t="inlineStr">
         <is>
           <t>0</t>
@@ -1501,7 +1426,7 @@
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>03-December-2025</t>
+          <t>03-March-2026</t>
         </is>
       </c>
       <c r="AC4" t="inlineStr">
@@ -1516,14 +1441,14 @@
       </c>
       <c r="AE4" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
           <t>930</t>
         </is>
       </c>
-      <c r="AF4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="AG4" t="inlineStr">
         <is>
           <t>0</t>
@@ -1541,7 +1466,7 @@
       </c>
       <c r="AK4" t="inlineStr">
         <is>
-          <t>02-December-2025</t>
+          <t>02-March-2026</t>
         </is>
       </c>
       <c r="AL4" t="inlineStr">
@@ -1583,32 +1508,32 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>08-December-2025</t>
+          <t>06-March-2026</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>pms</t>
+          <t>masterdata-eng</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>509</t>
+          <t>945</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>297</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>159</t>
+          <t>945</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -1618,17 +1543,17 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>05-December-2025</t>
+          <t>05-March-2026</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>masterdata-hin</t>
+          <t>masterdata-eng</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -1643,7 +1568,7 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>930</t>
+          <t>945</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -1653,7 +1578,7 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>0</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
@@ -1663,7 +1588,7 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>04-December-2025</t>
+          <t>04-March-2026</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -1678,14 +1603,14 @@
       </c>
       <c r="V5" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
           <t>945</t>
         </is>
       </c>
-      <c r="W5" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="X5" t="inlineStr">
         <is>
           <t>0</t>
@@ -1703,7 +1628,7 @@
       </c>
       <c r="AB5" t="inlineStr">
         <is>
-          <t>03-December-2025</t>
+          <t>03-March-2026</t>
         </is>
       </c>
       <c r="AC5" t="inlineStr">
@@ -1718,14 +1643,14 @@
       </c>
       <c r="AE5" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AF5" t="inlineStr">
+        <is>
           <t>945</t>
         </is>
       </c>
-      <c r="AF5" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="AG5" t="inlineStr">
         <is>
           <t>0</t>
@@ -1743,7 +1668,7 @@
       </c>
       <c r="AK5" t="inlineStr">
         <is>
-          <t>02-December-2025</t>
+          <t>02-March-2026</t>
         </is>
       </c>
       <c r="AL5" t="inlineStr">
@@ -1785,52 +1710,52 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>08-December-2025</t>
+          <t>06-March-2026</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>prereg</t>
+          <t>masterdata-fra</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>288</t>
+          <t>945</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>157</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>930</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>108</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>15</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>05-December-2025</t>
+          <t>05-March-2026</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>masterdata-kan</t>
+          <t>masterdata-fra</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -1865,7 +1790,7 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>04-December-2025</t>
+          <t>04-March-2026</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
@@ -1880,14 +1805,14 @@
       </c>
       <c r="V6" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
           <t>930</t>
         </is>
       </c>
-      <c r="W6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="X6" t="inlineStr">
         <is>
           <t>0</t>
@@ -1905,7 +1830,7 @@
       </c>
       <c r="AB6" t="inlineStr">
         <is>
-          <t>03-December-2025</t>
+          <t>03-March-2026</t>
         </is>
       </c>
       <c r="AC6" t="inlineStr">
@@ -1920,14 +1845,14 @@
       </c>
       <c r="AE6" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AF6" t="inlineStr">
+        <is>
           <t>930</t>
         </is>
       </c>
-      <c r="AF6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="AG6" t="inlineStr">
         <is>
           <t>0</t>
@@ -1945,7 +1870,7 @@
       </c>
       <c r="AK6" t="inlineStr">
         <is>
-          <t>02-December-2025</t>
+          <t>02-March-2026</t>
         </is>
       </c>
       <c r="AL6" t="inlineStr">
@@ -1987,182 +1912,182 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>08-December-2025</t>
+          <t>06-March-2026</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>dsl</t>
+          <t>pms</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>209</t>
+          <t>511</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
+          <t>487</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
           <t>4</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>35</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>135</t>
-        </is>
-      </c>
       <c r="G7" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
           <t>12</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
-      </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>05-December-2025</t>
+          <t>05-March-2026</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>masterdata-tam</t>
+          <t>pms</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>945</t>
+          <t>511</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>487</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>930</t>
+          <t>8</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>0</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>12</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>04-December-2025</t>
+          <t>04-March-2026</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>masterdata-hin</t>
+          <t>pms</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>945</t>
+          <t>511</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>930</t>
+          <t>487</t>
         </is>
       </c>
       <c r="W7" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>8</t>
         </is>
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
       <c r="Y7" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>0</t>
         </is>
       </c>
       <c r="Z7" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>12</t>
         </is>
       </c>
       <c r="AB7" t="inlineStr">
         <is>
-          <t>03-December-2025</t>
+          <t>03-March-2026</t>
         </is>
       </c>
       <c r="AC7" t="inlineStr">
         <is>
-          <t>masterdata-hin</t>
+          <t>pms</t>
         </is>
       </c>
       <c r="AD7" t="inlineStr">
         <is>
-          <t>945</t>
+          <t>511</t>
         </is>
       </c>
       <c r="AE7" t="inlineStr">
         <is>
-          <t>930</t>
+          <t>487</t>
         </is>
       </c>
       <c r="AF7" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AG7" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AH7" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AI7" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>12</t>
         </is>
       </c>
       <c r="AK7" t="inlineStr">
         <is>
-          <t>02-December-2025</t>
+          <t>02-March-2026</t>
         </is>
       </c>
       <c r="AL7" t="inlineStr">
         <is>
-          <t>masterdata-hin</t>
+          <t>pms</t>
         </is>
       </c>
       <c r="AM7" t="inlineStr">
         <is>
-          <t>945</t>
+          <t>511</t>
         </is>
       </c>
       <c r="AN7" t="inlineStr">
         <is>
-          <t>930</t>
+          <t>499</t>
         </is>
       </c>
       <c r="AO7" t="inlineStr">
@@ -2177,68 +2102,84 @@
       </c>
       <c r="AQ7" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AR7" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>12</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
-        <v/>
-      </c>
-      <c r="B8" t="n">
-        <v/>
-      </c>
-      <c r="C8" t="n">
-        <v/>
-      </c>
-      <c r="D8" t="n">
-        <v/>
-      </c>
-      <c r="E8" t="n">
-        <v/>
-      </c>
-      <c r="F8" t="n">
-        <v/>
-      </c>
-      <c r="G8" t="n">
-        <v/>
-      </c>
-      <c r="H8" t="n">
-        <v/>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>06-March-2026</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>prereg</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>288</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>284</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>05-December-2025</t>
+          <t>05-March-2026</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>pms</t>
+          <t>prereg</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>509</t>
+          <t>288</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>303</t>
+          <t>0</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>134</t>
+          <t>0</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>284</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -2248,27 +2189,27 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>4</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>04-December-2025</t>
+          <t>04-March-2026</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>masterdata-kan</t>
+          <t>prereg</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>945</t>
+          <t>288</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>930</t>
+          <t>0</t>
         </is>
       </c>
       <c r="W8" t="inlineStr">
@@ -2278,37 +2219,37 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>284</t>
         </is>
       </c>
       <c r="Y8" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>0</t>
         </is>
       </c>
       <c r="Z8" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AB8" t="inlineStr">
         <is>
-          <t>03-December-2025</t>
+          <t>03-March-2026</t>
         </is>
       </c>
       <c r="AC8" t="inlineStr">
         <is>
-          <t>masterdata-kan</t>
+          <t>prereg</t>
         </is>
       </c>
       <c r="AD8" t="inlineStr">
         <is>
-          <t>945</t>
+          <t>288</t>
         </is>
       </c>
       <c r="AE8" t="inlineStr">
         <is>
-          <t>930</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AF8" t="inlineStr">
@@ -2318,37 +2259,37 @@
       </c>
       <c r="AG8" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>284</t>
         </is>
       </c>
       <c r="AH8" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AI8" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AK8" t="inlineStr">
         <is>
-          <t>02-December-2025</t>
+          <t>02-March-2026</t>
         </is>
       </c>
       <c r="AL8" t="inlineStr">
         <is>
-          <t>masterdata-kan</t>
+          <t>prereg</t>
         </is>
       </c>
       <c r="AM8" t="inlineStr">
         <is>
-          <t>945</t>
+          <t>288</t>
         </is>
       </c>
       <c r="AN8" t="inlineStr">
         <is>
-          <t>930</t>
+          <t>282</t>
         </is>
       </c>
       <c r="AO8" t="inlineStr">
@@ -2363,73 +2304,89 @@
       </c>
       <c r="AQ8" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AR8" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
-        <v/>
-      </c>
-      <c r="B9" t="n">
-        <v/>
-      </c>
-      <c r="C9" t="n">
-        <v/>
-      </c>
-      <c r="D9" t="n">
-        <v/>
-      </c>
-      <c r="E9" t="n">
-        <v/>
-      </c>
-      <c r="F9" t="n">
-        <v/>
-      </c>
-      <c r="G9" t="n">
-        <v/>
-      </c>
-      <c r="H9" t="n">
-        <v/>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>06-March-2026</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>resident</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1142</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>1134</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>05-December-2025</t>
+          <t>05-March-2026</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>prereg</t>
+          <t>resident</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>288</t>
+          <t>1142</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>96</t>
+          <t>0</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>116</t>
+          <t>1134</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>74</t>
+          <t>8</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
@@ -2439,117 +2396,117 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>04-December-2025</t>
+          <t>04-March-2026</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>masterdata-tam</t>
+          <t>resident</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>945</t>
+          <t>1142</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>930</t>
+          <t>0</t>
         </is>
       </c>
       <c r="W9" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1134</t>
         </is>
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>8</t>
         </is>
       </c>
       <c r="Y9" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>03-March-2026</t>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>resident</t>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>1142</t>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AF9" t="inlineStr">
+        <is>
+          <t>1134</t>
+        </is>
+      </c>
+      <c r="AG9" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="AH9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AI9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AK9" t="inlineStr">
+        <is>
+          <t>02-March-2026</t>
+        </is>
+      </c>
+      <c r="AL9" t="inlineStr">
+        <is>
+          <t>resident</t>
+        </is>
+      </c>
+      <c r="AM9" t="inlineStr">
+        <is>
+          <t>1142</t>
+        </is>
+      </c>
+      <c r="AN9" t="inlineStr">
+        <is>
+          <t>1127</t>
+        </is>
+      </c>
+      <c r="AO9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AP9" t="inlineStr">
+        <is>
           <t>15</t>
         </is>
       </c>
-      <c r="Z9" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB9" t="inlineStr">
-        <is>
-          <t>03-December-2025</t>
-        </is>
-      </c>
-      <c r="AC9" t="inlineStr">
-        <is>
-          <t>masterdata-tam</t>
-        </is>
-      </c>
-      <c r="AD9" t="inlineStr">
-        <is>
-          <t>945</t>
-        </is>
-      </c>
-      <c r="AE9" t="inlineStr">
-        <is>
-          <t>930</t>
-        </is>
-      </c>
-      <c r="AF9" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AG9" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AH9" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="AI9" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AK9" t="inlineStr">
-        <is>
-          <t>02-December-2025</t>
-        </is>
-      </c>
-      <c r="AL9" t="inlineStr">
-        <is>
-          <t>masterdata-tam</t>
-        </is>
-      </c>
-      <c r="AM9" t="inlineStr">
-        <is>
-          <t>945</t>
-        </is>
-      </c>
-      <c r="AN9" t="inlineStr">
-        <is>
-          <t>930</t>
-        </is>
-      </c>
-      <c r="AO9" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AP9" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="AQ9" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AR9" t="inlineStr">
@@ -2559,33 +2516,49 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
-        <v/>
-      </c>
-      <c r="B10" t="n">
-        <v/>
-      </c>
-      <c r="C10" t="n">
-        <v/>
-      </c>
-      <c r="D10" t="n">
-        <v/>
-      </c>
-      <c r="E10" t="n">
-        <v/>
-      </c>
-      <c r="F10" t="n">
-        <v/>
-      </c>
-      <c r="G10" t="n">
-        <v/>
-      </c>
-      <c r="H10" t="n">
-        <v/>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>06-March-2026</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>dsl</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>209</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>179</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>05-December-2025</t>
+          <t>05-March-2026</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -2600,7 +2573,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -2610,7 +2583,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>173</t>
+          <t>179</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
@@ -2620,637 +2593,127 @@
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>18</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>04-December-2025</t>
+          <t>04-March-2026</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>pms</t>
+          <t>dsl</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>509</t>
+          <t>209</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>334</t>
+          <t>0</t>
         </is>
       </c>
       <c r="W10" t="inlineStr">
         <is>
-          <t>134</t>
+          <t>0</t>
         </is>
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>179</t>
         </is>
       </c>
       <c r="Y10" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>12</t>
         </is>
       </c>
       <c r="Z10" t="inlineStr">
         <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>03-March-2026</t>
+        </is>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>dsl</t>
+        </is>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>209</t>
+        </is>
+      </c>
+      <c r="AE10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AF10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AG10" t="inlineStr">
+        <is>
+          <t>179</t>
+        </is>
+      </c>
+      <c r="AH10" t="inlineStr">
+        <is>
           <t>12</t>
         </is>
       </c>
-      <c r="AB10" t="inlineStr">
-        <is>
-          <t>03-December-2025</t>
-        </is>
-      </c>
-      <c r="AC10" t="inlineStr">
-        <is>
-          <t>pms</t>
-        </is>
-      </c>
-      <c r="AD10" t="inlineStr">
-        <is>
-          <t>509</t>
-        </is>
-      </c>
-      <c r="AE10" t="inlineStr">
-        <is>
-          <t>334</t>
-        </is>
-      </c>
-      <c r="AF10" t="inlineStr">
-        <is>
-          <t>134</t>
-        </is>
-      </c>
-      <c r="AG10" t="inlineStr">
-        <is>
-          <t>29</t>
-        </is>
-      </c>
-      <c r="AH10" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="AI10" t="inlineStr">
         <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="AK10" t="inlineStr">
+        <is>
+          <t>02-March-2026</t>
+        </is>
+      </c>
+      <c r="AL10" t="inlineStr">
+        <is>
+          <t>dsl</t>
+        </is>
+      </c>
+      <c r="AM10" t="inlineStr">
+        <is>
+          <t>209</t>
+        </is>
+      </c>
+      <c r="AN10" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="AO10" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="AP10" t="inlineStr">
+        <is>
+          <t>79</t>
+        </is>
+      </c>
+      <c r="AQ10" t="inlineStr">
+        <is>
           <t>12</t>
         </is>
       </c>
-      <c r="AK10" t="inlineStr">
-        <is>
-          <t>02-December-2025</t>
-        </is>
-      </c>
-      <c r="AL10" t="inlineStr">
-        <is>
-          <t>pms</t>
-        </is>
-      </c>
-      <c r="AM10" t="inlineStr">
-        <is>
-          <t>509</t>
-        </is>
-      </c>
-      <c r="AN10" t="inlineStr">
-        <is>
-          <t>334</t>
-        </is>
-      </c>
-      <c r="AO10" t="inlineStr">
-        <is>
-          <t>134</t>
-        </is>
-      </c>
-      <c r="AP10" t="inlineStr">
-        <is>
-          <t>29</t>
-        </is>
-      </c>
-      <c r="AQ10" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="AR10" t="inlineStr">
         <is>
-          <t>12</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v/>
-      </c>
-      <c r="B11" t="n">
-        <v/>
-      </c>
-      <c r="C11" t="n">
-        <v/>
-      </c>
-      <c r="D11" t="n">
-        <v/>
-      </c>
-      <c r="E11" t="n">
-        <v/>
-      </c>
-      <c r="F11" t="n">
-        <v/>
-      </c>
-      <c r="G11" t="n">
-        <v/>
-      </c>
-      <c r="H11" t="n">
-        <v/>
-      </c>
-      <c r="J11" t="n">
-        <v/>
-      </c>
-      <c r="K11" t="n">
-        <v/>
-      </c>
-      <c r="L11" t="n">
-        <v/>
-      </c>
-      <c r="M11" t="n">
-        <v/>
-      </c>
-      <c r="N11" t="n">
-        <v/>
-      </c>
-      <c r="O11" t="n">
-        <v/>
-      </c>
-      <c r="P11" t="n">
-        <v/>
-      </c>
-      <c r="Q11" t="n">
-        <v/>
-      </c>
-      <c r="S11" t="inlineStr">
-        <is>
-          <t>04-December-2025</t>
-        </is>
-      </c>
-      <c r="T11" t="inlineStr">
-        <is>
-          <t>prereg</t>
-        </is>
-      </c>
-      <c r="U11" t="inlineStr">
-        <is>
-          <t>288</t>
-        </is>
-      </c>
-      <c r="V11" t="inlineStr">
-        <is>
-          <t>219</t>
-        </is>
-      </c>
-      <c r="W11" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="X11" t="inlineStr">
-        <is>
-          <t>63</t>
-        </is>
-      </c>
-      <c r="Y11" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="Z11" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB11" t="inlineStr">
-        <is>
-          <t>03-December-2025</t>
-        </is>
-      </c>
-      <c r="AC11" t="inlineStr">
-        <is>
-          <t>prereg</t>
-        </is>
-      </c>
-      <c r="AD11" t="inlineStr">
-        <is>
-          <t>288</t>
-        </is>
-      </c>
-      <c r="AE11" t="inlineStr">
-        <is>
-          <t>219</t>
-        </is>
-      </c>
-      <c r="AF11" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="AG11" t="inlineStr">
-        <is>
-          <t>63</t>
-        </is>
-      </c>
-      <c r="AH11" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="AI11" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AK11" t="inlineStr">
-        <is>
-          <t>02-December-2025</t>
-        </is>
-      </c>
-      <c r="AL11" t="inlineStr">
-        <is>
-          <t>prereg</t>
-        </is>
-      </c>
-      <c r="AM11" t="inlineStr">
-        <is>
-          <t>288</t>
-        </is>
-      </c>
-      <c r="AN11" t="inlineStr">
-        <is>
-          <t>219</t>
-        </is>
-      </c>
-      <c r="AO11" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="AP11" t="inlineStr">
-        <is>
-          <t>63</t>
-        </is>
-      </c>
-      <c r="AQ11" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="AR11" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v/>
-      </c>
-      <c r="B12" t="n">
-        <v/>
-      </c>
-      <c r="C12" t="n">
-        <v/>
-      </c>
-      <c r="D12" t="n">
-        <v/>
-      </c>
-      <c r="E12" t="n">
-        <v/>
-      </c>
-      <c r="F12" t="n">
-        <v/>
-      </c>
-      <c r="G12" t="n">
-        <v/>
-      </c>
-      <c r="H12" t="n">
-        <v/>
-      </c>
-      <c r="J12" t="n">
-        <v/>
-      </c>
-      <c r="K12" t="n">
-        <v/>
-      </c>
-      <c r="L12" t="n">
-        <v/>
-      </c>
-      <c r="M12" t="n">
-        <v/>
-      </c>
-      <c r="N12" t="n">
-        <v/>
-      </c>
-      <c r="O12" t="n">
-        <v/>
-      </c>
-      <c r="P12" t="n">
-        <v/>
-      </c>
-      <c r="Q12" t="n">
-        <v/>
-      </c>
-      <c r="S12" t="inlineStr">
-        <is>
-          <t>04-December-2025</t>
-        </is>
-      </c>
-      <c r="T12" t="inlineStr">
-        <is>
-          <t>resident</t>
-        </is>
-      </c>
-      <c r="U12" t="inlineStr">
-        <is>
-          <t>1124</t>
-        </is>
-      </c>
-      <c r="V12" t="inlineStr">
-        <is>
-          <t>1109</t>
-        </is>
-      </c>
-      <c r="W12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="X12" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="Y12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="Z12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB12" t="inlineStr">
-        <is>
-          <t>03-December-2025</t>
-        </is>
-      </c>
-      <c r="AC12" t="inlineStr">
-        <is>
-          <t>resident</t>
-        </is>
-      </c>
-      <c r="AD12" t="inlineStr">
-        <is>
-          <t>1124</t>
-        </is>
-      </c>
-      <c r="AE12" t="inlineStr">
-        <is>
-          <t>1115</t>
-        </is>
-      </c>
-      <c r="AF12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AG12" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="AH12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AI12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AK12" t="inlineStr">
-        <is>
-          <t>02-December-2025</t>
-        </is>
-      </c>
-      <c r="AL12" t="inlineStr">
-        <is>
-          <t>resident</t>
-        </is>
-      </c>
-      <c r="AM12" t="inlineStr">
-        <is>
-          <t>1124</t>
-        </is>
-      </c>
-      <c r="AN12" t="inlineStr">
-        <is>
-          <t>1109</t>
-        </is>
-      </c>
-      <c r="AO12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AP12" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="AQ12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AR12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v/>
-      </c>
-      <c r="B13" t="n">
-        <v/>
-      </c>
-      <c r="C13" t="n">
-        <v/>
-      </c>
-      <c r="D13" t="n">
-        <v/>
-      </c>
-      <c r="E13" t="n">
-        <v/>
-      </c>
-      <c r="F13" t="n">
-        <v/>
-      </c>
-      <c r="G13" t="n">
-        <v/>
-      </c>
-      <c r="H13" t="n">
-        <v/>
-      </c>
-      <c r="J13" t="n">
-        <v/>
-      </c>
-      <c r="K13" t="n">
-        <v/>
-      </c>
-      <c r="L13" t="n">
-        <v/>
-      </c>
-      <c r="M13" t="n">
-        <v/>
-      </c>
-      <c r="N13" t="n">
-        <v/>
-      </c>
-      <c r="O13" t="n">
-        <v/>
-      </c>
-      <c r="P13" t="n">
-        <v/>
-      </c>
-      <c r="Q13" t="n">
-        <v/>
-      </c>
-      <c r="S13" t="inlineStr">
-        <is>
-          <t>04-December-2025</t>
-        </is>
-      </c>
-      <c r="T13" t="inlineStr">
-        <is>
-          <t>dsl</t>
-        </is>
-      </c>
-      <c r="U13" t="inlineStr">
-        <is>
-          <t>210</t>
-        </is>
-      </c>
-      <c r="V13" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="W13" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="X13" t="inlineStr">
-        <is>
-          <t>168</t>
-        </is>
-      </c>
-      <c r="Y13" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="Z13" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
-      <c r="AB13" t="inlineStr">
-        <is>
-          <t>03-December-2025</t>
-        </is>
-      </c>
-      <c r="AC13" t="inlineStr">
-        <is>
-          <t>dsl</t>
-        </is>
-      </c>
-      <c r="AD13" t="inlineStr">
-        <is>
-          <t>210</t>
-        </is>
-      </c>
-      <c r="AE13" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="AF13" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AG13" t="inlineStr">
-        <is>
-          <t>163</t>
-        </is>
-      </c>
-      <c r="AH13" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="AI13" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
-      <c r="AK13" t="inlineStr">
-        <is>
-          <t>02-December-2025</t>
-        </is>
-      </c>
-      <c r="AL13" t="inlineStr">
-        <is>
-          <t>dsl</t>
-        </is>
-      </c>
-      <c r="AM13" t="inlineStr">
-        <is>
-          <t>210</t>
-        </is>
-      </c>
-      <c r="AN13" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="AO13" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AP13" t="inlineStr">
-        <is>
-          <t>169</t>
-        </is>
-      </c>
-      <c r="AQ13" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="AR13" t="inlineStr">
-        <is>
-          <t>24</t>
+          <t>18</t>
         </is>
       </c>
     </row>

</xml_diff>